<commit_message>
Nowe nazewnictwo: FG / FR01–FR13 dla ryflowań, kody typów FGN, FGP, FGO, FGOP, EGL
Stare kody ryflowań (F00, F01…) z zapisanych koszyków i linków są przeliczane na nowe.
Cennik w Excelu, README i pytania do szefa zaktualizowane.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q5tgYXGzQjFTT1Be5g96Bb
</commit_message>
<xml_diff>
--- a/docs/cennik-fronty-giete.xlsx
+++ b/docs/cennik-fronty-giete.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Cennik" sheetId="1" state="visible" r:id="rId3"/>
@@ -35,16 +35,16 @@
     <t xml:space="preserve">Materiał</t>
   </si>
   <si>
-    <t xml:space="preserve">Gładki (F00) [zł/m²]</t>
+    <t xml:space="preserve">Gładki (FG) [zł/m²]</t>
   </si>
   <si>
     <t xml:space="preserve">Ryflowany [zł/m²]</t>
   </si>
   <si>
-    <t xml:space="preserve">F07 [zł/m²]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F08 [zł/m²]</t>
+    <t xml:space="preserve">FR07 [zł/m²]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FR08 [zł/m²]</t>
   </si>
   <si>
     <t xml:space="preserve">Uwagi</t>
@@ -59,7 +59,7 @@
     <t xml:space="preserve">Fornirowane</t>
   </si>
   <si>
-    <t xml:space="preserve">Do ustalenia z szefem (gładki / ryflowany / F07–F08).</t>
+    <t xml:space="preserve">Do ustalenia z szefem (gładki / ryflowany / FR07–FR08).</t>
   </si>
   <si>
     <t xml:space="preserve">Laminat</t>
@@ -125,85 +125,85 @@
     <t xml:space="preserve">Laminat [zł/m²]</t>
   </si>
   <si>
-    <t xml:space="preserve">F00</t>
+    <t xml:space="preserve">FG</t>
   </si>
   <si>
     <t xml:space="preserve">Gładki</t>
   </si>
   <si>
-    <t xml:space="preserve">F01</t>
+    <t xml:space="preserve">FR01</t>
   </si>
   <si>
     <t xml:space="preserve">Wpust 15</t>
   </si>
   <si>
-    <t xml:space="preserve">F02</t>
+    <t xml:space="preserve">FR02</t>
   </si>
   <si>
     <t xml:space="preserve">Klin 15</t>
   </si>
   <si>
-    <t xml:space="preserve">F03</t>
+    <t xml:space="preserve">FR03</t>
   </si>
   <si>
     <t xml:space="preserve">Fala 18</t>
   </si>
   <si>
-    <t xml:space="preserve">F04</t>
+    <t xml:space="preserve">FR04</t>
   </si>
   <si>
     <t xml:space="preserve">Fala 12</t>
   </si>
   <si>
-    <t xml:space="preserve">F05</t>
+    <t xml:space="preserve">FR05</t>
   </si>
   <si>
     <t xml:space="preserve">Wałek 19</t>
   </si>
   <si>
-    <t xml:space="preserve">F06</t>
+    <t xml:space="preserve">FR06</t>
   </si>
   <si>
     <t xml:space="preserve">Wałek 25</t>
   </si>
   <si>
-    <t xml:space="preserve">F07</t>
+    <t xml:space="preserve">FR07</t>
   </si>
   <si>
     <t xml:space="preserve">Wałek 9</t>
   </si>
   <si>
-    <t xml:space="preserve">F08</t>
+    <t xml:space="preserve">FR08</t>
   </si>
   <si>
     <t xml:space="preserve">Wpust 20</t>
   </si>
   <si>
-    <t xml:space="preserve">F09</t>
+    <t xml:space="preserve">FR09</t>
   </si>
   <si>
     <t xml:space="preserve">Rowek 6</t>
   </si>
   <si>
-    <t xml:space="preserve">F10</t>
+    <t xml:space="preserve">FR10</t>
   </si>
   <si>
     <t xml:space="preserve">Rowek 3</t>
   </si>
   <si>
-    <t xml:space="preserve">F11</t>
+    <t xml:space="preserve">FR11</t>
   </si>
   <si>
     <t xml:space="preserve">Wpust 10</t>
   </si>
   <si>
-    <t xml:space="preserve">F12</t>
+    <t xml:space="preserve">FR12</t>
   </si>
   <si>
     <t xml:space="preserve">Fala 10</t>
   </si>
   <si>
-    <t xml:space="preserve">F13</t>
+    <t xml:space="preserve">FR13</t>
   </si>
   <si>
     <t xml:space="preserve">Klin 10</t>
@@ -242,7 +242,7 @@
     <t xml:space="preserve">Przedłużenia lewe/prawe: 0 lub 10–50 mm (0 i 0 → N0, jedno → N1, oba → N2)</t>
   </si>
   <si>
-    <t xml:space="preserve">EG-N0/N1/N2-R###</t>
+    <t xml:space="preserve">FGN-N0/N1/N2-R###</t>
   </si>
   <si>
     <t xml:space="preserve">Przedłużane</t>
@@ -254,7 +254,7 @@
     <t xml:space="preserve">L = od lica łuku do końca: R+50 … 700 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">EG-N1-R###-L###</t>
+    <t xml:space="preserve">FGP-R###-L###</t>
   </si>
   <si>
     <t xml:space="preserve">Obustronne</t>
@@ -269,7 +269,7 @@
     <t xml:space="preserve">W = 600 / 700 / 800 mm; boki Z: brak lub R+10 … 200 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">EG-D-R100-W###[-Z###]</t>
+    <t xml:space="preserve">FGO-R100-W### (z bokami Z: FGOP-R100-W###-Z###)</t>
   </si>
   <si>
     <t xml:space="preserve">W łuk</t>
@@ -284,7 +284,7 @@
     <t xml:space="preserve">—</t>
   </si>
   <si>
-    <t xml:space="preserve">EG-P-R###</t>
+    <t xml:space="preserve">EGL-R###</t>
   </si>
   <si>
     <t xml:space="preserve">Wymiary ogólne</t>
@@ -329,7 +329,7 @@
     <t xml:space="preserve">Ograniczenia</t>
   </si>
   <si>
-    <t xml:space="preserve">Tylko gładki (F00)</t>
+    <t xml:space="preserve">Tylko gładki (FG)</t>
   </si>
   <si>
     <t xml:space="preserve">Opcjonalny (dekor)</t>
@@ -338,7 +338,7 @@
     <t xml:space="preserve">Jedyny materiał przy H &gt; 2780 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">Wszystkie F00–F13</t>
+    <t xml:space="preserve">Wszystkie FG, FR01–FR13</t>
   </si>
   <si>
     <t xml:space="preserve">Opcjonalny (np. dąb, bejca)</t>
@@ -392,7 +392,7 @@
     <t xml:space="preserve">Kalkulator wyceny jednej pozycji</t>
   </si>
   <si>
-    <t xml:space="preserve">Wpisz / wybierz wartości w niebieskich komórkach (kolumna B). Przykład poniżej: narożny R300, H 720, przedłużenia 30/40, lakier F07, bryła, 2 szt.</t>
+    <t xml:space="preserve">Wpisz / wybierz wartości w niebieskich komórkach (kolumna B). Przykład poniżej: narożny R300, H 720, przedłużenia 30/40, lakier FR07, bryła, 2 szt.</t>
   </si>
   <si>
     <t xml:space="preserve">Dane wejściowe</t>
@@ -443,7 +443,7 @@
     <t xml:space="preserve">Laminat / Fornirowane / Lakierowane</t>
   </si>
   <si>
-    <t xml:space="preserve">F00–F13 (laminat zawsze F00)</t>
+    <t xml:space="preserve">FG, FR01–FR13 (laminat zawsze FG)</t>
   </si>
   <si>
     <t xml:space="preserve">Bryła (TAK/NIE)</t>
@@ -533,7 +533,7 @@
     <t xml:space="preserve">Odpowiedź (do uzupełnienia)</t>
   </si>
   <si>
-    <t xml:space="preserve">Fornir – ile za m²? Gładki / ryflowany? Czy F07 i F08 też droższe?</t>
+    <t xml:space="preserve">Fornir – ile za m²? Gładki / ryflowany? Czy FR07 i FR08 też droższe?</t>
   </si>
   <si>
     <t xml:space="preserve">Laminat – ile za m² (tylko gładki)? To jedyny materiał przy H &gt; 2780 mm.</t>
@@ -2281,8 +2281,8 @@
         <v>152</v>
       </c>
       <c r="B23" s="20" t="str">
-        <f aca="false">IF(B13="Laminat","F00",B14)</f>
-        <v>F07</v>
+        <f aca="false">IF(B13="Laminat","FG",B14)</f>
+        <v>FR07</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>153</v>

</xml_diff>